<commit_message>
security(privacy): anonymize tracked sample spreadsheets with zero-PII realistic mock data for public repository
</commit_message>
<xml_diff>
--- a/Prod/candidates_tracker.xlsx
+++ b/Prod/candidates_tracker.xlsx
@@ -587,17 +587,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ashwin Rasquinha</t>
+          <t>Priya Patel 01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>+91 98868 95438 / +91 91776 89177 / 08762441712</t>
+          <t>+91 98765 00001</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>rasquinha.ashwin@gmail.com</t>
+          <t>priyapatel01@example.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -610,9 +610,6 @@
           <t>Extracted from PDF</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>Actively Looking</t>
@@ -623,26 +620,21 @@
           <t>LinkedIn</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr"/>
+          <t>+91 98765 00000:13:06</t>
+        </is>
+      </c>
       <c r="N2" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>Android mobile verified at 00:27:52: Box items scroll and fit screen perfectly.</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
       <c r="S2" t="inlineStr">
         <is>
           <t>L2 - Raj</t>
@@ -658,27 +650,21 @@
           <t>Escalated to L2 Raj: Review candidate Python experience and suggest compensation.</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
-      <c r="Y2" t="inlineStr"/>
-      <c r="Z2" t="inlineStr"/>
-      <c r="AA2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SASMITA HEMBRAM</t>
+          <t>Rohan Verma 02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>+91 9061676594</t>
+          <t>+91 98765 00002</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>sasmitahembram56@gmail.com</t>
+          <t>rohanverma02@example.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -703,7 +689,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -725,17 +711,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Sukanya</t>
+          <t>Ananya Iyer 03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>+91 9000685614</t>
+          <t>+91 98765 00003</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sukanyasukanya99981@gmail.com</t>
+          <t>ananyaiyer03@example.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -755,7 +741,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -777,17 +763,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ARBHAZ PASHA M</t>
+          <t>Vikram Malhotra 04</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>+91-9743455404, 701934912</t>
+          <t>+91 98765 00004</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>arbhazpasham@gmail.com</t>
+          <t>vikrammalhotra04@example.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -812,7 +798,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -822,7 +808,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -834,17 +820,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GANEASHA SUBRAMANIAN</t>
+          <t>Neha Gupta 05</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>+91 8310625634</t>
+          <t>+91 98765 00005</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ganeasha.subramanian@gmail.com</t>
+          <t>nehagupta05@example.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -869,7 +855,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -881,17 +867,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SNEH JANGRA</t>
+          <t>Siddharth Rao 06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>+91 9311739491</t>
+          <t>+91 98765 00006</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Jangra.sneh@gmail.com</t>
+          <t>siddharthrao06@example.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -916,7 +902,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -928,17 +914,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>PRASHANTH K. C</t>
+          <t>Kavita Nair 07</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>8618443570</t>
+          <t>+91 98765 00007</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>kaloseprashanth@rediffmail.com</t>
+          <t>kavitanair07@example.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -963,7 +949,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -973,7 +959,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
@@ -985,17 +971,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Sangamesh G S</t>
+          <t>Aditya Joshi 08</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>9481667211</t>
+          <t>+91 98765 00008</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>officersangamesh99@gmail.com</t>
+          <t>adityajoshi08@example.com</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1020,7 +1006,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1030,7 +1016,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
@@ -1042,17 +1028,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SAM LI JOSE A</t>
+          <t>Pooja Reddy 09</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>8892534537</t>
+          <t>+91 98765 00009</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Samlijose28@gmail.com</t>
+          <t>poojareddy09@example.com</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1077,7 +1063,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1087,7 +1073,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -1099,17 +1085,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Shilpa M</t>
+          <t>Rajesh Pillai 10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>+91 9901298470</t>
+          <t>+91 98765 00010</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>shilpa9071002410@gmail.com</t>
+          <t>rajeshpillai10@example.com</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1134,7 +1120,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1144,7 +1130,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1156,17 +1142,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SNEHA MARY J</t>
+          <t>Sunita Deshmukh 11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>6363238567</t>
+          <t>+91 98765 00011</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>snehavijay767@gmai.com</t>
+          <t>sunitadeshmukh11@example.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1191,7 +1177,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1201,7 +1187,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1213,17 +1199,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Karankumar</t>
+          <t>Arjun Kapoor 12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>+91 9916166008</t>
+          <t>+91 98765 00012</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>karanbablad3655@gmail.com</t>
+          <t>arjunkapoor12@example.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1248,7 +1234,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1258,7 +1244,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1270,17 +1256,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABHISHEK. N.</t>
+          <t>Meera Bhattacharya 13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>8310209994</t>
+          <t>+91 98765 00013</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>abhishek09268mahi@gmail.com</t>
+          <t>meerabhattacharya13@example.com</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1305,7 +1291,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1315,7 +1301,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -1327,17 +1313,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BHARATH L</t>
+          <t>Karan Mehra 14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6363625189</t>
+          <t>+91 98765 00014</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>bharathloki97@gmail.com</t>
+          <t>karanmehra14@example.com</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1362,7 +1348,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -1372,7 +1358,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -1384,17 +1370,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MAHESHWARI R</t>
+          <t>Deepika Saxena 15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>9739697240</t>
+          <t>+91 98765 00015</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>mahiraju52146@gmail.com.</t>
+          <t>deepikasaxena15@example.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1419,7 +1405,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -1429,7 +1415,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
@@ -1446,17 +1432,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Shilpa C</t>
+          <t>Suresh Menon 16</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>9738085420</t>
+          <t>+91 98765 00016</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Shilpaclement96@gmail.com</t>
+          <t>sureshmenon16@example.com</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1481,7 +1467,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -1491,7 +1477,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
@@ -1503,17 +1489,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SAI YESWANTH PESALA</t>
+          <t>Divya Chawla 17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>+91 9100410784</t>
+          <t>+91 98765 00017</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>yaswanthyashsai@gmail.com</t>
+          <t>divyachawla17@example.com</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1538,7 +1524,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -1548,7 +1534,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
@@ -1560,17 +1546,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LESTER JOHNSON GOVEAS</t>
+          <t>Manoj Kulkarni 18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>9482835605</t>
+          <t>+91 98765 00018</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>lestergoveas1@gmail.com</t>
+          <t>manojkulkarni18@example.com</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1595,7 +1581,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -1605,7 +1591,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>+91 98765 00000</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
@@ -1617,17 +1603,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>NILESH KUMAR SINHA</t>
+          <t>Swati Sen 19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>+91-8249558366</t>
+          <t>+91 98765 00019</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>nileshks.connect@gmail.com</t>
+          <t>swatisen19@example.com</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1652,7 +1638,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>2026-08-22 19:13:06</t>
+          <t>+91 98765 00000:13:06</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -1664,17 +1650,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TRACEY MIESEL</t>
+          <t>Nikhil Chatterjee 20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>(886) 834-8215</t>
+          <t>+91 98765 00020</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>tracey.miesel@gmail.com</t>
+          <t>nikhilchatterjee20@example.com</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1699,7 +1685,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -1711,17 +1697,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PRASHANT KUMAR PRASAD</t>
+          <t>Bhavna Jain 21</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>+91 8083555868</t>
+          <t>+91 98765 00021</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>kr.prashant94@gmail.com</t>
+          <t>bhavnajain21@example.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1746,7 +1732,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -1758,17 +1744,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Kishan Kumar</t>
+          <t>Gaurav Das 22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>+91 98765 00022</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>hello@kishans.in</t>
+          <t>gauravdas22@example.com</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1793,7 +1779,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -1805,17 +1791,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Anirudh Maiya</t>
+          <t>Tanvi Singhal 23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>(720) 314-2147</t>
+          <t>+91 98765 00023</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>anirudhmaiya99@gmail.com</t>
+          <t>tanvisinghal23@example.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1840,7 +1826,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -1852,17 +1838,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Muhammad Ghulam Jillani</t>
+          <t>Amit Trivedi 24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>+92-321-1174167</t>
+          <t>+91 98765 00024</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>m.g.jillani123@gmail.com</t>
+          <t>amittrivedi24@example.com</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1887,7 +1873,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -1899,17 +1885,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Shreyas Puttaraju</t>
+          <t>Aarav Sharma 25</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>224-389-0281</t>
+          <t>+91 98765 00025</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>shreyas2797@gmail.com</t>
+          <t>aaravsharma25@example.com</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1934,7 +1920,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -1946,17 +1932,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Pranshul Kushwaha</t>
+          <t>Priya Patel 26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>202601-0833</t>
+          <t>+91 98765 00026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>priyapatel26@example.com</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1981,7 +1967,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
@@ -1993,17 +1979,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Amit Kumar Pundhir</t>
+          <t>Rohan Verma 27</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>+91 98765 00027</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>rohanverma27@example.com</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -2028,7 +2014,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
@@ -2040,17 +2026,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Mallikarjun HM</t>
+          <t>Ananya Iyer 28</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>+91 98765 00028</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Not Found</t>
+          <t>ananyaiyer28@example.com</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2075,7 +2061,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
@@ -2087,17 +2073,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Corrinda Andoh</t>
+          <t>Vikram Malhotra 29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>(421) 407-5566</t>
+          <t>+91 98765 00029</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>corrinda.andoh@gmail.com</t>
+          <t>vikrammalhotra29@example.com</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -2122,7 +2108,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -2134,17 +2120,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Group Captain Ajit Kumar Sinha</t>
+          <t>Neha Gupta 30</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>+91-8875018933</t>
+          <t>+91 98765 00030</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>nehagupta30@example.com</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -2184,7 +2170,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -2196,17 +2182,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Rakesh Iyer Sp</t>
+          <t>Siddharth Rao 31</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>+91-7204458839</t>
+          <t>+91 98765 00031</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>siddharthrao31@example.com</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2246,7 +2232,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -2258,17 +2244,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Colonel Kapil Dev Patel</t>
+          <t>Kavita Nair 32</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>+91-9933939596</t>
+          <t>+91 98765 00032</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>kavitanair32@example.com</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2308,7 +2294,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -2320,17 +2306,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Sanjay Balodhi</t>
+          <t>Aditya Joshi 33</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>+91-8368868357</t>
+          <t>+91 98765 00033</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>adityajoshi33@example.com</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2370,7 +2356,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -2382,17 +2368,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Maschendra Yadav</t>
+          <t>Pooja Reddy 34</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>+91-9036398842</t>
+          <t>+91 98765 00034</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>poojareddy34@example.com</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2432,7 +2418,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -2444,17 +2430,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Rohit Subhash Patil</t>
+          <t>Rajesh Pillai 35</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>+91-9916510989</t>
+          <t>+91 98765 00035</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>rajeshpillai35@example.com</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2494,7 +2480,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -2506,17 +2492,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Palaksha Kn</t>
+          <t>Sunita Deshmukh 36</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>+91-9731552050</t>
+          <t>+91 98765 00036</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>sunitadeshmukh36@example.com</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2556,7 +2542,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -2568,17 +2554,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Radha Krishan Sharma</t>
+          <t>Arjun Kapoor 37</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>+91-8278618712</t>
+          <t>+91 98765 00037</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>arjunkapoor37@example.com</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2618,7 +2604,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
@@ -2630,17 +2616,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Rajdeep Mishra</t>
+          <t>Meera Bhattacharya 38</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>+91-8449950520</t>
+          <t>+91 98765 00038</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>meerabhattacharya38@example.com</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2680,7 +2666,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
@@ -2692,17 +2678,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Vijaya Kumar Varaganti</t>
+          <t>Karan Mehra 39</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>+91-9966882641</t>
+          <t>+91 98765 00039</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>karanmehra39@example.com</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2742,7 +2728,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
@@ -2754,17 +2740,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Anshul Kanwe</t>
+          <t>Deepika Saxena 40</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>+91-9893302662</t>
+          <t>+91 98765 00040</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>deepikasaxena40@example.com</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2804,7 +2790,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
@@ -2816,17 +2802,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Harsh Vardhan Sharma</t>
+          <t>Suresh Menon 41</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>+91-7001927746</t>
+          <t>+91 98765 00041</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>sureshmenon41@example.com</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2866,7 +2852,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
@@ -2878,17 +2864,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Sounak Babeja</t>
+          <t>Divya Chawla 42</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>+91-8906546235</t>
+          <t>+91 98765 00042</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>divyachawla42@example.com</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2928,7 +2914,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
@@ -2940,17 +2926,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>S Radhakrishnan</t>
+          <t>Manoj Kulkarni 43</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>+91-8861302761</t>
+          <t>+91 98765 00043</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>manojkulkarni43@example.com</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2990,7 +2976,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
@@ -3002,17 +2988,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Ramanathan Thiyagarajan</t>
+          <t>Swati Sen 44</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>+91-7200743228</t>
+          <t>+91 98765 00044</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>swatisen44@example.com</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -3052,7 +3038,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
@@ -3064,17 +3050,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Tanvi Bhatnagar</t>
+          <t>Nikhil Chatterjee 45</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>+91-9611398009</t>
+          <t>+91 98765 00045</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>nikhilchatterjee45@example.com</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -3114,7 +3100,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
@@ -3126,17 +3112,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Shubhang Shukla</t>
+          <t>Bhavna Jain 46</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>+91-9454997109</t>
+          <t>+91 98765 00046</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>bhavnajain46@example.com</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -3176,7 +3162,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
@@ -3188,17 +3174,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Vasanth Kumar Panibhate</t>
+          <t>Gaurav Das 47</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>+91-7975506609</t>
+          <t>+91 98765 00047</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>gauravdas47@example.com</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -3238,7 +3224,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
@@ -3250,17 +3236,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Pavithra H R</t>
+          <t>Tanvi Singhal 48</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>+91-9972036686</t>
+          <t>+91 98765 00048</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>tanvisinghal48@example.com</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -3300,7 +3286,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
@@ -3312,17 +3298,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Bakul Joshi</t>
+          <t>Amit Trivedi 49</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>+91-9545405449</t>
+          <t>+91 98765 00049</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>amittrivedi49@example.com</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -3362,7 +3348,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N50" t="inlineStr">
@@ -3374,17 +3360,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Asha B S</t>
+          <t>Aarav Sharma 50</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>+91-9880484345</t>
+          <t>+91 98765 00050</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>aaravsharma50@example.com</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3424,7 +3410,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N51" t="inlineStr">
@@ -3436,17 +3422,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Chotan Kumar</t>
+          <t>Priya Patel 51</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>+91-7676750267</t>
+          <t>+91 98765 00051</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>priyapatel51@example.com</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -3486,7 +3472,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N52" t="inlineStr">
@@ -3498,17 +3484,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Nancy Ronald</t>
+          <t>Rohan Verma 52</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>+91-9620797976</t>
+          <t>+91 98765 00052</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>rohanverma52@example.com</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -3548,7 +3534,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N53" t="inlineStr">
@@ -3560,17 +3546,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Sunil</t>
+          <t>Ananya Iyer 53</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>+65-9620963888</t>
+          <t>+91 98765 00053</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>ananyaiyer53@example.com</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -3610,7 +3596,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N54" t="inlineStr">
@@ -3622,17 +3608,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Vishvanath A V</t>
+          <t>Vikram Malhotra 54</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>+91-9739915517</t>
+          <t>+91 98765 00054</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>vikrammalhotra54@example.com</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -3672,7 +3658,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N55" t="inlineStr">
@@ -3684,17 +3670,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Ravi Shalavadi</t>
+          <t>Neha Gupta 55</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>+91-8904195713</t>
+          <t>+91 98765 00055</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>nehagupta55@example.com</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -3734,7 +3720,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N56" t="inlineStr">
@@ -3746,17 +3732,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Prashanth Arakere Mayanna</t>
+          <t>Siddharth Rao 56</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>+91-9886744462</t>
+          <t>+91 98765 00056</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>siddharthrao56@example.com</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -3796,7 +3782,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N57" t="inlineStr">
@@ -3808,17 +3794,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Nandakumar N</t>
+          <t>Kavita Nair 57</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>+91-9886858281</t>
+          <t>+91 98765 00057</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>kavitanair57@example.com</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -3858,7 +3844,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N58" t="inlineStr">
@@ -3870,17 +3856,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Bhoomika R Pawar</t>
+          <t>Aditya Joshi 58</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>+91-9916291572</t>
+          <t>+91 98765 00058</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>adityajoshi58@example.com</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -3920,7 +3906,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N59" t="inlineStr">
@@ -3932,17 +3918,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Jeevan B K</t>
+          <t>Pooja Reddy 59</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>+91-7204410471</t>
+          <t>+91 98765 00059</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>poojareddy59@example.com</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -3982,7 +3968,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N60" t="inlineStr">
@@ -3994,17 +3980,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Ranbijay Kumar</t>
+          <t>Rajesh Pillai 60</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>+91-9810602725</t>
+          <t>+91 98765 00060</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>rajeshpillai60@example.com</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -4044,7 +4030,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N61" t="inlineStr">
@@ -4056,17 +4042,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Prashant Halijol</t>
+          <t>Sunita Deshmukh 61</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>+91-7204583830</t>
+          <t>+91 98765 00061</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>sunitadeshmukh61@example.com</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -4106,7 +4092,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N62" t="inlineStr">
@@ -4118,17 +4104,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Software Engineer (Snowflake Developer)</t>
+          <t>Arjun Kapoor 62</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>+91-7095709438</t>
+          <t>+91 98765 00062</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>arjunkapoor62@example.com</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -4168,7 +4154,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N63" t="inlineStr">
@@ -4180,17 +4166,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Prasanna Ganapathi S</t>
+          <t>Meera Bhattacharya 63</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>+91-6360453743</t>
+          <t>+91 98765 00063</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>meerabhattacharya63@example.com</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -4230,7 +4216,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N64" t="inlineStr">
@@ -4242,17 +4228,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Vinodkumar V S</t>
+          <t>Karan Mehra 64</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>+91-6362245944</t>
+          <t>+91 98765 00064</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>karanmehra64@example.com</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -4292,7 +4278,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N65" t="inlineStr">
@@ -4304,17 +4290,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Gopi R R</t>
+          <t>Deepika Saxena 65</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>+91-8884223345</t>
+          <t>+91 98765 00065</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>deepikasaxena65@example.com</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -4354,7 +4340,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N66" t="inlineStr">
@@ -4366,17 +4352,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Sundeep Joshi</t>
+          <t>Suresh Menon 66</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>+91-9597738267</t>
+          <t>+91 98765 00066</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>sureshmenon66@example.com</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -4416,7 +4402,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N67" t="inlineStr">
@@ -4428,17 +4414,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Sandeep Kumar</t>
+          <t>Divya Chawla 67</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>+91-8884072225</t>
+          <t>+91 98765 00067</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>divyachawla67@example.com</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -4478,7 +4464,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N68" t="inlineStr">
@@ -4490,17 +4476,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Rapur Ramya</t>
+          <t>Manoj Kulkarni 68</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>+91-7989466489</t>
+          <t>+91 98765 00068</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>manojkulkarni68@example.com</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -4540,7 +4526,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N69" t="inlineStr">
@@ -4552,17 +4538,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Balaji M</t>
+          <t>Swati Sen 69</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>+91-9014648663</t>
+          <t>+91 98765 00069</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>swatisen69@example.com</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4602,7 +4588,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N70" t="inlineStr">
@@ -4614,17 +4600,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Subedar Shivakumar G J</t>
+          <t>Nikhil Chatterjee 70</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>+91-9483471780</t>
+          <t>+91 98765 00070</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>nikhilchatterjee70@example.com</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4664,7 +4650,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N71" t="inlineStr">
@@ -4676,17 +4662,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Ravikumar Nimmalapalli</t>
+          <t>Bhavna Jain 71</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>+91-7358302017</t>
+          <t>+91 98765 00071</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>bhavnajain71@example.com</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4726,7 +4712,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N72" t="inlineStr">
@@ -4738,17 +4724,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Manoranjan Dash</t>
+          <t>Gaurav Das 72</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>+91-9480436392</t>
+          <t>+91 98765 00072</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>gauravdas72@example.com</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4788,7 +4774,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N73" t="inlineStr">
@@ -4800,17 +4786,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Mysore Ranganath</t>
+          <t>Tanvi Singhal 73</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>+91-8951239709</t>
+          <t>+91 98765 00073</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>tanvisinghal73@example.com</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -4850,7 +4836,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N74" t="inlineStr">
@@ -4862,17 +4848,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Shashidhar S</t>
+          <t>Amit Trivedi 74</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>+91-9900092815</t>
+          <t>+91 98765 00074</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>amittrivedi74@example.com</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -4912,7 +4898,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N75" t="inlineStr">
@@ -4924,17 +4910,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Sathyanarayana Maiya</t>
+          <t>Aarav Sharma 75</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>+91-9449613411</t>
+          <t>+91 98765 00075</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>aaravsharma75@example.com</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -4974,7 +4960,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N76" t="inlineStr">
@@ -4986,17 +4972,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Sriram</t>
+          <t>Priya Patel 76</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>+91-9741188717</t>
+          <t>+91 98765 00076</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>priyapatel76@example.com</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -5036,7 +5022,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N77" t="inlineStr">
@@ -5048,17 +5034,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Amarnarayana Manchinbale</t>
+          <t>Rohan Verma 77</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>+91-9945344417</t>
+          <t>+91 98765 00077</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>rohanverma77@example.com</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -5098,7 +5084,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N78" t="inlineStr">
@@ -5110,17 +5096,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Debasis Saha</t>
+          <t>Ananya Iyer 78</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>+91-9980843809</t>
+          <t>+91 98765 00078</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>ananyaiyer78@example.com</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -5160,7 +5146,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N79" t="inlineStr">
@@ -5172,17 +5158,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Ramesh Kumar Dhar</t>
+          <t>Vikram Malhotra 79</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>+91-9425403824</t>
+          <t>+91 98765 00079</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>vikrammalhotra79@example.com</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -5222,7 +5208,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N80" t="inlineStr">
@@ -5234,17 +5220,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Kiran Kumar</t>
+          <t>Neha Gupta 80</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>+91-9483504599</t>
+          <t>+91 98765 00080</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>nehagupta80@example.com</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -5284,7 +5270,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N81" t="inlineStr">
@@ -5296,17 +5282,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Subramany</t>
+          <t>Siddharth Rao 81</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>+91 98765 00081</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>subramanygopala@...</t>
+          <t>siddharthrao81@example.com</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -5346,7 +5332,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N82" t="inlineStr">
@@ -5358,17 +5344,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Bindu Sunil</t>
+          <t>Kavita Nair 82</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>+91-8848127443</t>
+          <t>+91 98765 00082</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>kavitanair82@example.com</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -5408,7 +5394,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N83" t="inlineStr">
@@ -5420,17 +5406,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Bhanumathi Balasubramanian</t>
+          <t>Aditya Joshi 83</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>+91-9833980137</t>
+          <t>+91 98765 00083</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>adityajoshi83@example.com</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -5470,7 +5456,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N84" t="inlineStr">
@@ -5482,17 +5468,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Harish Chourasia</t>
+          <t>Pooja Reddy 84</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>+91-9425042413</t>
+          <t>+91 98765 00084</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>poojareddy84@example.com</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -5532,7 +5518,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N85" t="inlineStr">
@@ -5544,17 +5530,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Raunak Sharma</t>
+          <t>Rajesh Pillai 85</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>+91-8800772888</t>
+          <t>+91 98765 00085</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>rajeshpillai85@example.com</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -5594,7 +5580,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
@@ -5606,17 +5592,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Motupalli Sekhar Chitikela</t>
+          <t>Sunita Deshmukh 86</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>+91-9986040456</t>
+          <t>+91 98765 00086</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>sunitadeshmukh86@example.com</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -5656,7 +5642,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
@@ -5668,17 +5654,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Sudhir Dubey</t>
+          <t>Arjun Kapoor 87</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>+91-9971892335</t>
+          <t>+91 98765 00087</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>arjunkapoor87@example.com</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -5718,7 +5704,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
@@ -5730,17 +5716,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Bhavani Shankar V</t>
+          <t>Meera Bhattacharya 88</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>+91-9740376397</t>
+          <t>+91 98765 00088</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>meerabhattacharya88@example.com</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -5780,7 +5766,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N89" t="inlineStr">
@@ -5792,17 +5778,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>V. Hariharan Hariharan</t>
+          <t>Karan Mehra 89</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>+91-9500042605</t>
+          <t>+91 98765 00089</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>karanmehra89@example.com</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -5842,7 +5828,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N90" t="inlineStr">
@@ -5854,17 +5840,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Ramakrishna Rao</t>
+          <t>Deepika Saxena 90</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>+91-8310791068</t>
+          <t>+91 98765 00090</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>deepikasaxena90@example.com</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -5904,7 +5890,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
@@ -5916,17 +5902,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Rajesh Upadhyay</t>
+          <t>Suresh Menon 91</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>+91-9884917438</t>
+          <t>+91 98765 00091</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>sureshmenon91@example.com</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -5966,7 +5952,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N92" t="inlineStr">
@@ -5978,17 +5964,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Karan Singh</t>
+          <t>Divya Chawla 92</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>+91-7395092462</t>
+          <t>+91 98765 00092</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>divyachawla92@example.com</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -6028,7 +6014,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N93" t="inlineStr">
@@ -6040,17 +6026,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Balamurugan R</t>
+          <t>Manoj Kulkarni 93</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>+91-8122588291</t>
+          <t>+91 98765 00093</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>manojkulkarni93@example.com</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -6090,7 +6076,7 @@
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
@@ -6102,17 +6088,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Raju</t>
+          <t>Swati Sen 94</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>+91-7795043068</t>
+          <t>+91 98765 00094</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>swatisen94@example.com</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -6152,7 +6138,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N95" t="inlineStr">
@@ -6164,17 +6150,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Nilanjana Roy</t>
+          <t>Nikhil Chatterjee 95</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>+91-9830547737</t>
+          <t>+91 98765 00095</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>nikhilchatterjee95@example.com</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -6214,7 +6200,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N96" t="inlineStr">
@@ -6226,17 +6212,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Rajesh Walia</t>
+          <t>Bhavna Jain 96</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>+91-9779585883</t>
+          <t>+91 98765 00096</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>bhavnajain96@example.com</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -6276,7 +6262,7 @@
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N97" t="inlineStr">
@@ -6288,17 +6274,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Angad Singh</t>
+          <t>Gaurav Das 97</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>+91-8867493457</t>
+          <t>+91 98765 00097</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>gauravdas97@example.com</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -6338,7 +6324,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N98" t="inlineStr">
@@ -6350,17 +6336,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Krishna Kumar U</t>
+          <t>Tanvi Singhal 98</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>+91-8660342492</t>
+          <t>+91 98765 00098</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>tanvisinghal98@example.com</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -6400,7 +6386,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N99" t="inlineStr">
@@ -6412,17 +6398,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Subramanian Ananthanarayanan</t>
+          <t>Amit Trivedi 99</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>+91-9902168702</t>
+          <t>+91 98765 00099</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>amittrivedi99@example.com</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -6462,7 +6448,7 @@
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N100" t="inlineStr">
@@ -6474,17 +6460,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Jayakumar J</t>
+          <t>Aarav Sharma 100</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>+91-9444900288</t>
+          <t>+91 98765 00100</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>aaravsharma100@example.com</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -6524,7 +6510,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N101" t="inlineStr">
@@ -6536,17 +6522,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Milind Kulabkar</t>
+          <t>Priya Patel 101</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>+91-9740545522</t>
+          <t>+91 98765 00101</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>priyapatel101@example.com</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -6586,7 +6572,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N102" t="inlineStr">
@@ -6598,17 +6584,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Sudhir Venugopal</t>
+          <t>Rohan Verma 102</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>+91-8884316596</t>
+          <t>+91 98765 00102</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>rohanverma102@example.com</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -6648,7 +6634,7 @@
       </c>
       <c r="L103" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N103" t="inlineStr">
@@ -6660,17 +6646,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Ghais Moula Bakhshuddin</t>
+          <t>Ananya Iyer 103</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>+91-9483545910</t>
+          <t>+91 98765 00103</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>ananyaiyer103@example.com</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -6710,7 +6696,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N104" t="inlineStr">
@@ -6722,17 +6708,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>A Udaya Bhaskar Reddy</t>
+          <t>Vikram Malhotra 104</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>+91-7032913704</t>
+          <t>+91 98765 00104</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>vikrammalhotra104@example.com</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -6772,7 +6758,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
@@ -6784,17 +6770,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Sundeep Trehan</t>
+          <t>Neha Gupta 105</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>+91-9845159108</t>
+          <t>+91 98765 00105</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>nehagupta105@example.com</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -6834,7 +6820,7 @@
       </c>
       <c r="L106" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N106" t="inlineStr">
@@ -6846,17 +6832,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Columnist Retired (CR)</t>
+          <t>Siddharth Rao 106</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>+91-8670370915</t>
+          <t>+91 98765 00106</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>siddharthrao106@example.com</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -6896,7 +6882,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N107" t="inlineStr">
@@ -6908,17 +6894,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Jogindra Prasad Prajapati</t>
+          <t>Kavita Nair 107</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>+91-8431469172</t>
+          <t>+91 98765 00107</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>kavitanair107@example.com</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -6958,7 +6944,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N108" t="inlineStr">
@@ -6970,17 +6956,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Chakravarthi Mohan IAS Retired</t>
+          <t>Aditya Joshi 108</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>+91-9740615317</t>
+          <t>+91 98765 00108</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>adityajoshi108@example.com</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
@@ -7020,7 +7006,7 @@
       </c>
       <c r="L109" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N109" t="inlineStr">
@@ -7032,17 +7018,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Gururaj</t>
+          <t>Pooja Reddy 109</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>+91-9148983479</t>
+          <t>+91 98765 00109</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>poojareddy109@example.com</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -7082,7 +7068,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N110" t="inlineStr">
@@ -7094,17 +7080,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Uday Kulkarni</t>
+          <t>Rajesh Pillai 110</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>+91-8431317725</t>
+          <t>+91 98765 00110</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>rajeshpillai110@example.com</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -7144,7 +7130,7 @@
       </c>
       <c r="L111" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N111" t="inlineStr">
@@ -7156,17 +7142,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Mark Louis TPR</t>
+          <t>Sunita Deshmukh 111</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>+91-9902732716</t>
+          <t>+91 98765 00111</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>sunitadeshmukh111@example.com</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -7206,7 +7192,7 @@
       </c>
       <c r="L112" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N112" t="inlineStr">
@@ -7218,17 +7204,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Udaya Kumar</t>
+          <t>Arjun Kapoor 112</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>+91 98765 00112</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>udayakumarc@rediffmail.com</t>
+          <t>arjunkapoor112@example.com</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -7268,7 +7254,7 @@
       </c>
       <c r="L113" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N113" t="inlineStr">
@@ -7280,17 +7266,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Narendranath Krishnan Menon</t>
+          <t>Meera Bhattacharya 113</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>+91-9611028028</t>
+          <t>+91 98765 00113</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>meerabhattacharya113@example.com</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -7330,7 +7316,7 @@
       </c>
       <c r="L114" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N114" t="inlineStr">
@@ -7342,17 +7328,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Bobby Abraham</t>
+          <t>Karan Mehra 114</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>+91-9663177712</t>
+          <t>+91 98765 00114</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>karanmehra114@example.com</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -7392,7 +7378,7 @@
       </c>
       <c r="L115" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N115" t="inlineStr">
@@ -7404,17 +7390,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Sales Head / Client Relations Manager (SA)</t>
+          <t>Deepika Saxena 115</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>+91-9739935959</t>
+          <t>+91 98765 00115</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>deepikasaxena115@example.com</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -7454,7 +7440,7 @@
       </c>
       <c r="L116" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N116" t="inlineStr">
@@ -7466,17 +7452,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Lakshmi Bhat</t>
+          <t>Suresh Menon 116</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>+91-9845592108</t>
+          <t>+91 98765 00116</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>sureshmenon116@example.com</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -7516,7 +7502,7 @@
       </c>
       <c r="L117" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N117" t="inlineStr">
@@ -7528,17 +7514,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Kunhiraman Chirammal</t>
+          <t>Divya Chawla 117</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>+91-8848642154</t>
+          <t>+91 98765 00117</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>divyachawla117@example.com</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -7578,7 +7564,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N118" t="inlineStr">
@@ -7590,17 +7576,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>N D Guru Prasad</t>
+          <t>Manoj Kulkarni 118</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>+91-9343824343</t>
+          <t>+91 98765 00118</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>manojkulkarni118@example.com</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -7640,7 +7626,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N119" t="inlineStr">
@@ -7652,17 +7638,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Gokul</t>
+          <t>Swati Sen 119</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>+91-9438133308</t>
+          <t>+91 98765 00119</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>swatisen119@example.com</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -7702,7 +7688,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N120" t="inlineStr">
@@ -7714,17 +7700,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Santhosh Kumar Manghat</t>
+          <t>Nikhil Chatterjee 120</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>+91-9986044386</t>
+          <t>+91 98765 00120</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>nikhilchatterjee120@example.com</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -7764,7 +7750,7 @@
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N121" t="inlineStr">
@@ -7776,17 +7762,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Govindan Iyer</t>
+          <t>Bhavna Jain 121</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>+91-9900577554</t>
+          <t>+91 98765 00121</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>bhavnajain121@example.com</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
@@ -7826,7 +7812,7 @@
       </c>
       <c r="L122" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N122" t="inlineStr">
@@ -7838,17 +7824,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Madhusudanan K B</t>
+          <t>Gaurav Das 122</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>+91-9900950384</t>
+          <t>+91 98765 00122</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>gauravdas122@example.com</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -7888,7 +7874,7 @@
       </c>
       <c r="L123" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N123" t="inlineStr">
@@ -7900,17 +7886,17 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Gopakumar</t>
+          <t>Tanvi Singhal 123</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>+91-8891297160</t>
+          <t>+91 98765 00123</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>tanvisinghal123@example.com</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -7950,7 +7936,7 @@
       </c>
       <c r="L124" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N124" t="inlineStr">
@@ -7962,17 +7948,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Sapna Singh</t>
+          <t>Amit Trivedi 124</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>+91 98765 00124</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>amittrivedi124@example.com</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
@@ -7997,7 +7983,7 @@
       </c>
       <c r="L125" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N125" t="inlineStr">
@@ -8009,17 +7995,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Masud Alam</t>
+          <t>Aarav Sharma 125</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>+91 98765 00125</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>Not Available</t>
+          <t>aaravsharma125@example.com</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -8044,7 +8030,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N126" t="inlineStr">
@@ -8056,17 +8042,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Pravin Agrawal</t>
+          <t>Priya Patel 126</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>+91-7890000000 (View Number)</t>
+          <t>+91 98765 00126</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>priyapatel126@example.com</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -8091,7 +8077,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N127" t="inlineStr">
@@ -8103,17 +8089,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Narayana Rao</t>
+          <t>Rohan Verma 127</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>+91-9730000000 (View Number)</t>
+          <t>+91 98765 00127</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>rohanverma127@example.com</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -8138,7 +8124,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N128" t="inlineStr">
@@ -8150,17 +8136,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Ranjan Gaming</t>
+          <t>Ananya Iyer 128</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>+91-8960000000 (View Number)</t>
+          <t>+91 98765 00128</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>ananyaiyer128@example.com</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -8185,7 +8171,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N129" t="inlineStr">
@@ -8197,17 +8183,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Ram</t>
+          <t>Vikram Malhotra 129</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>+91-9090000000 (View Number)</t>
+          <t>+91 98765 00129</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Verified phone</t>
+          <t>vikrammalhotra129@example.com</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -8247,7 +8233,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N130" t="inlineStr">
@@ -8259,17 +8245,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Eeri</t>
+          <t>Neha Gupta 130</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>+91-7880000000 (View Number)</t>
+          <t>+91 98765 00130</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Verified email id</t>
+          <t>nehagupta130@example.com</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
@@ -8294,7 +8280,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>2026-08-30 23:31:42</t>
+          <t>+91 98765 00000:31:42</t>
         </is>
       </c>
       <c r="N131" t="inlineStr">

</xml_diff>